<commit_message>
fix: corrige fechamento mensal e seleção de competência
</commit_message>
<xml_diff>
--- a/exports/relatorio_comissao.xlsx
+++ b/exports/relatorio_comissao.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$L$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,15 +459,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
@@ -805,47 +805,959 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="4" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>283.05</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>226.44</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>28.31</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>177.35</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>141.88</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>17.73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>178.9</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>143.12</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>17.89</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>46214</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>350.6</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>280.48</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>35.06</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>311.6</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>249.28</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>31.16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>129.35</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>103.48</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>12.94</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>170.4</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>136.32</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>17.04</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>202.3</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>161.84</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>23.12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>235</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>26.86</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>346.8</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>277.44</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>39.63</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>320.1</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>256.08</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>32.01</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>46222</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>168.9</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>135.12</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>16.89</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>245.05</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>196.04</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>24.51</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>222.95</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>178.36</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="J22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="L22" s="5" t="n">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>229.4</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>183.52</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>22.94</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>233.9</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>187.12</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="K24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>23.39</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>262.05</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>209.64</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+      <c r="L25" s="5" t="n">
+        <v>26.21</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>549.4</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>439.52</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="J26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="K26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+      <c r="L26" s="5" t="n">
+        <v>54.94</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>329.55</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>263.64</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>29.29</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>182.85</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>146.28</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>16.25</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>176.15</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>140.92</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>15.66</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>244.1</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>195.28</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>21.7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>348.75</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>279</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>34.88</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>261.75</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>209.4</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>26.18</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>1209.25</v>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>967.4</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>84.65000000000001</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="I9" s="7" t="n">
-        <v>102.65</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>81.73999999999999</v>
-      </c>
-      <c r="K9" s="7" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>116.4</v>
+      <c r="B33" s="7" t="n">
+        <v>7369.5</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>5895.6</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>228.61</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>733.3</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>643.6900000000001</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>733.3</v>
+      </c>
+      <c r="H33" s="7" t="n">
+        <v>733.3</v>
+      </c>
+      <c r="I33" s="7" t="n">
+        <v>719.55</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>637.58</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>733.3</v>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>733.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>